<commit_message>
Introduce heuristics weights in objective function
Introduce heuristics weights in objective function
</commit_message>
<xml_diff>
--- a/test/production/20260309-20260405/result.xlsx
+++ b/test/production/20260309-20260405/result.xlsx
@@ -282,7 +282,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="15">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1"/>
     <xf fontId="1" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
@@ -294,13 +294,10 @@
     <xf fontId="1" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf fontId="2" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
     <xf fontId="2" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1"/>
+    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf fontId="3" fillId="0" borderId="1" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf fontId="2" fillId="0" borderId="2" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
     <xf fontId="2" fillId="0" borderId="3" numFmtId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="2" numFmtId="0" xfId="0" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1"/>
-    <xf fontId="3" fillId="0" borderId="0" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -961,22 +958,22 @@
       <c r="I2" t="s">
         <v>39</v>
       </c>
-      <c r="J2" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="K2" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="L2" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="M2" s="11" t="s">
+      <c r="J2" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="K2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="L2" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="M2" s="4" t="s">
         <v>42</v>
       </c>
       <c r="N2" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="O2" s="12" t="s">
+      <c r="O2" s="1" t="s">
         <v>40</v>
       </c>
       <c r="P2" t="s">
@@ -1072,22 +1069,22 @@
       <c r="I3" t="s">
         <v>39</v>
       </c>
-      <c r="J3" s="11" t="s">
+      <c r="J3" s="4" t="s">
         <v>38</v>
       </c>
       <c r="K3" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="L3" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="M3" s="11" t="s">
+      <c r="L3" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="M3" s="4" t="s">
         <v>39</v>
       </c>
       <c r="N3" t="s">
         <v>41</v>
       </c>
-      <c r="O3" s="12" t="s">
+      <c r="O3" s="1" t="s">
         <v>38</v>
       </c>
       <c r="P3" t="s">
@@ -1168,37 +1165,37 @@
       <c r="D4" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="E4" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="F4" s="9" t="s">
+      <c r="E4" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="F4" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="G4" s="9" t="s">
-        <v>38</v>
-      </c>
-      <c r="H4" s="10" t="s">
-        <v>40</v>
-      </c>
-      <c r="I4" t="s">
-        <v>40</v>
-      </c>
-      <c r="J4" s="2" t="s">
+      <c r="G4" s="11" t="s">
+        <v>38</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="I4" s="11" t="s">
+        <v>40</v>
+      </c>
+      <c r="J4" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="K4" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="L4" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="M4" s="11" t="s">
+      <c r="K4" s="11" t="s">
+        <v>39</v>
+      </c>
+      <c r="L4" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="M4" s="4" t="s">
         <v>40</v>
       </c>
       <c r="N4" t="s">
         <v>40</v>
       </c>
-      <c r="O4" s="12" t="s">
+      <c r="O4" s="1" t="s">
         <v>39</v>
       </c>
       <c r="P4" t="s">
@@ -1294,22 +1291,22 @@
       <c r="I5" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="J5" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="K5" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="L5" s="15" t="s">
+      <c r="J5" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="K5" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="L5" s="5" t="s">
         <v>39</v>
       </c>
       <c r="M5" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="N5" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="O5" s="16" t="s">
+      <c r="N5" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="O5" s="6" t="s">
         <v>39</v>
       </c>
       <c r="P5" s="7" t="s">
@@ -1357,7 +1354,7 @@
       <c r="AD5" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="AE5" s="15" t="s">
+      <c r="AE5" s="5" t="s">
         <v>41</v>
       </c>
       <c r="AF5" s="7" t="s">
@@ -1422,13 +1419,13 @@
       <c r="L6" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="M6" s="11" t="s">
+      <c r="M6" s="4" t="s">
         <v>39</v>
       </c>
       <c r="N6" t="s">
         <v>39</v>
       </c>
-      <c r="O6" s="12" t="s">
+      <c r="O6" s="1" t="s">
         <v>39</v>
       </c>
       <c r="P6" t="s">
@@ -1527,19 +1524,19 @@
       <c r="J7" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="K7" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="L7" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="M7" s="11" t="s">
+      <c r="K7" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="L7" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="M7" s="4" t="s">
         <v>39</v>
       </c>
       <c r="N7" t="s">
         <v>42</v>
       </c>
-      <c r="O7" s="12" t="s">
+      <c r="O7" s="1" t="s">
         <v>39</v>
       </c>
       <c r="P7" t="s">
@@ -1635,22 +1632,22 @@
       <c r="I8" t="s">
         <v>39</v>
       </c>
-      <c r="J8" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="K8" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="L8" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="M8" s="11" t="s">
+      <c r="J8" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="K8" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="L8" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="M8" s="4" t="s">
         <v>40</v>
       </c>
       <c r="N8" t="s">
         <v>40</v>
       </c>
-      <c r="O8" s="12" t="s">
+      <c r="O8" s="1" t="s">
         <v>38</v>
       </c>
       <c r="P8" t="s">
@@ -1695,13 +1692,13 @@
       <c r="AC8" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="AD8" t="s">
+      <c r="AD8" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="AE8" t="s">
-        <v>40</v>
-      </c>
-      <c r="AF8" t="s">
+      <c r="AE8" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="AF8" s="2" t="s">
         <v>40</v>
       </c>
       <c r="AG8" s="2" t="s">
@@ -1743,7 +1740,7 @@
       <c r="H9" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="I9" s="15" t="s">
+      <c r="I9" s="5" t="s">
         <v>40</v>
       </c>
       <c r="J9" s="7" t="s">
@@ -1752,16 +1749,16 @@
       <c r="K9" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="L9" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="M9" s="15" t="s">
+      <c r="L9" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="M9" s="5" t="s">
         <v>38</v>
       </c>
       <c r="N9" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="O9" s="16" t="s">
+      <c r="O9" s="6" t="s">
         <v>40</v>
       </c>
       <c r="P9" s="7" t="s">
@@ -1866,16 +1863,16 @@
       <c r="I10" t="s">
         <v>42</v>
       </c>
-      <c r="J10" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="K10" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="L10" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="M10" s="11" t="s">
+      <c r="J10" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="K10" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="L10" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="M10" s="4" t="s">
         <v>39</v>
       </c>
       <c r="N10" t="s">
@@ -1947,8 +1944,8 @@
       <c r="AJ10" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="AK10" s="17"/>
-      <c r="AL10" s="17"/>
+      <c r="AK10" s="11"/>
+      <c r="AL10" s="11"/>
     </row>
     <row r="11" ht="14.25">
       <c r="A11" t="s">
@@ -1978,13 +1975,13 @@
       <c r="I11" t="s">
         <v>39</v>
       </c>
-      <c r="J11" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="K11" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="L11" s="11" t="s">
+      <c r="J11" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="K11" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="L11" s="4" t="s">
         <v>39</v>
       </c>
       <c r="M11" s="2" t="s">
@@ -1993,7 +1990,7 @@
       <c r="N11" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="O11" s="12" t="s">
+      <c r="O11" s="1" t="s">
         <v>40</v>
       </c>
       <c r="P11" t="s">
@@ -2089,22 +2086,22 @@
       <c r="I12" t="s">
         <v>40</v>
       </c>
-      <c r="J12" s="11" t="s">
+      <c r="J12" s="4" t="s">
         <v>40</v>
       </c>
       <c r="K12" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="L12" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="M12" s="11" t="s">
+      <c r="L12" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="M12" s="4" t="s">
         <v>38</v>
       </c>
       <c r="N12" t="s">
         <v>40</v>
       </c>
-      <c r="O12" s="12" t="s">
+      <c r="O12" s="1" t="s">
         <v>42</v>
       </c>
       <c r="P12" t="s">
@@ -2197,25 +2194,25 @@
       <c r="H13" s="14" t="s">
         <v>39</v>
       </c>
-      <c r="I13" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="J13" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="K13" s="15" t="s">
+      <c r="I13" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="J13" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="K13" s="5" t="s">
         <v>42</v>
       </c>
       <c r="L13" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="M13" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="N13" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="O13" s="16" t="s">
+      <c r="M13" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="N13" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="O13" s="6" t="s">
         <v>39</v>
       </c>
       <c r="P13" s="7" t="s">
@@ -2311,22 +2308,22 @@
       <c r="I14" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="J14" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="K14" s="11" t="s">
-        <v>38</v>
-      </c>
-      <c r="L14" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="M14" s="11" t="s">
+      <c r="J14" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="K14" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="L14" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="M14" s="4" t="s">
         <v>40</v>
       </c>
       <c r="N14" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="O14" s="12" t="s">
+      <c r="O14" s="1" t="s">
         <v>39</v>
       </c>
       <c r="P14" t="s">
@@ -2422,22 +2419,22 @@
       <c r="I15" t="s">
         <v>39</v>
       </c>
-      <c r="J15" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="K15" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="L15" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="M15" s="11" t="s">
+      <c r="J15" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="K15" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="L15" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="M15" s="4" t="s">
         <v>39</v>
       </c>
       <c r="N15" t="s">
         <v>39</v>
       </c>
-      <c r="O15" s="12" t="s">
+      <c r="O15" s="1" t="s">
         <v>39</v>
       </c>
       <c r="P15" s="2" t="s">
@@ -2503,8 +2500,8 @@
       <c r="AJ15" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="AK15" s="17"/>
-      <c r="AL15" s="17"/>
+      <c r="AK15" s="11"/>
+      <c r="AL15" s="11"/>
     </row>
     <row r="16" ht="14.25">
       <c r="A16" t="s">
@@ -2534,22 +2531,22 @@
       <c r="I16" t="s">
         <v>38</v>
       </c>
-      <c r="J16" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="K16" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="L16" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="M16" s="11" t="s">
+      <c r="J16" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="K16" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="L16" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="M16" s="4" t="s">
         <v>39</v>
       </c>
       <c r="N16" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="O16" s="12" t="s">
+      <c r="O16" s="1" t="s">
         <v>40</v>
       </c>
       <c r="P16" t="s">
@@ -2642,19 +2639,19 @@
       <c r="H17" s="14" t="s">
         <v>38</v>
       </c>
-      <c r="I17" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="J17" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="K17" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="L17" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="M17" s="15" t="s">
+      <c r="I17" s="5" t="s">
+        <v>40</v>
+      </c>
+      <c r="J17" s="5" t="s">
+        <v>42</v>
+      </c>
+      <c r="K17" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="L17" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="M17" s="5" t="s">
         <v>38</v>
       </c>
       <c r="N17" s="7" t="s">
@@ -2756,13 +2753,13 @@
       <c r="I18" t="s">
         <v>39</v>
       </c>
-      <c r="J18" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="K18" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="L18" s="11" t="s">
+      <c r="J18" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="K18" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="L18" s="4" t="s">
         <v>42</v>
       </c>
       <c r="M18" s="2" t="s">
@@ -2771,7 +2768,7 @@
       <c r="N18" t="s">
         <v>39</v>
       </c>
-      <c r="O18" s="12" t="s">
+      <c r="O18" s="1" t="s">
         <v>42</v>
       </c>
       <c r="P18" t="s">
@@ -2867,22 +2864,22 @@
       <c r="I19" t="s">
         <v>39</v>
       </c>
-      <c r="J19" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="K19" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="L19" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="M19" s="11" t="s">
+      <c r="J19" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="K19" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="L19" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="M19" s="4" t="s">
         <v>39</v>
       </c>
       <c r="N19" t="s">
         <v>42</v>
       </c>
-      <c r="O19" s="12" t="s">
+      <c r="O19" s="1" t="s">
         <v>42</v>
       </c>
       <c r="P19" t="s">
@@ -2978,22 +2975,22 @@
       <c r="I20" t="s">
         <v>42</v>
       </c>
-      <c r="J20" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="K20" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="L20" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="M20" s="11" t="s">
+      <c r="J20" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="K20" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="L20" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="M20" s="4" t="s">
         <v>42</v>
       </c>
       <c r="N20" t="s">
         <v>39</v>
       </c>
-      <c r="O20" s="12" t="s">
+      <c r="O20" s="1" t="s">
         <v>39</v>
       </c>
       <c r="P20" t="s">
@@ -3092,19 +3089,19 @@
       <c r="J21" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="K21" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="L21" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="M21" s="11" t="s">
+      <c r="K21" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="L21" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="M21" s="4" t="s">
         <v>42</v>
       </c>
       <c r="N21" t="s">
         <v>42</v>
       </c>
-      <c r="O21" s="12" t="s">
+      <c r="O21" s="1" t="s">
         <v>39</v>
       </c>
       <c r="P21" t="s">

</xml_diff>